<commit_message>
chore(radar): auto audit update 2026-09-08
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M178"/>
+  <dimension ref="A1:M188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10867,7 +10867,655 @@
         </is>
       </c>
     </row>
-    <row r="178"/>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>718.36</v>
+      </c>
+      <c r="D178" t="n">
+        <v>-0.0008</v>
+      </c>
+      <c r="E178" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="F178" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>225.73</v>
+      </c>
+      <c r="D179" t="n">
+        <v>-0.0201</v>
+      </c>
+      <c r="E179" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="F179" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>316.22</v>
+      </c>
+      <c r="D180" t="n">
+        <v>-0.0117</v>
+      </c>
+      <c r="E180" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F180" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>493.95</v>
+      </c>
+      <c r="D181" t="n">
+        <v>-0.0115</v>
+      </c>
+      <c r="E181" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="F181" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>256.97</v>
+      </c>
+      <c r="D182" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="E182" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F182" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>613.48</v>
+      </c>
+      <c r="D183" t="n">
+        <v>-0.0053</v>
+      </c>
+      <c r="E183" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="F183" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>RVol: 1.14x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>338.36</v>
+      </c>
+      <c r="D184" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="E184" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="F184" t="n">
+        <v>1</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>368.16</v>
+      </c>
+      <c r="D185" t="n">
+        <v>0.0398</v>
+      </c>
+      <c r="E185" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="F185" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>RVol: 1.34x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>1000.26</v>
+      </c>
+      <c r="D186" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="E186" t="n">
+        <v>43.45</v>
+      </c>
+      <c r="F186" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>477.3</v>
+      </c>
+      <c r="D187" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="E187" t="n">
+        <v>24.66</v>
+      </c>
+      <c r="F187" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>904.38</v>
+      </c>
+      <c r="D188" t="n">
+        <v>0.0649</v>
+      </c>
+      <c r="E188" t="n">
+        <v>65.43000000000001</v>
+      </c>
+      <c r="F188" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>RVol: 1.38x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-09
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M188"/>
+  <dimension ref="A1:M199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11516,6 +11516,655 @@
         </is>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>716.3099999999999</v>
+      </c>
+      <c r="D189" t="n">
+        <v>-0.0029</v>
+      </c>
+      <c r="E189" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="F189" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>223.67</v>
+      </c>
+      <c r="D190" t="n">
+        <v>-0.0091</v>
+      </c>
+      <c r="E190" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="F190" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>RVol: 0.61x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>315.34</v>
+      </c>
+      <c r="D191" t="n">
+        <v>-0.0028</v>
+      </c>
+      <c r="E191" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="F191" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>RVol: 1.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>491.65</v>
+      </c>
+      <c r="D192" t="n">
+        <v>-0.004699999999999999</v>
+      </c>
+      <c r="E192" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F192" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>RVol: 0.57x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>252.4</v>
+      </c>
+      <c r="D193" t="n">
+        <v>-0.0178</v>
+      </c>
+      <c r="E193" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F193" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>653.6900000000001</v>
+      </c>
+      <c r="D194" t="n">
+        <v>0.0655</v>
+      </c>
+      <c r="E194" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="F194" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>RVol: 2.18x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>330.65</v>
+      </c>
+      <c r="D195" t="n">
+        <v>-0.0228</v>
+      </c>
+      <c r="E195" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="F195" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>RVol: 1.46x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>367.81</v>
+      </c>
+      <c r="D196" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="E196" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="F196" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>1027.77</v>
+      </c>
+      <c r="D197" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="E197" t="n">
+        <v>50.11</v>
+      </c>
+      <c r="F197" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>482.28</v>
+      </c>
+      <c r="D198" t="n">
+        <v>0.0104</v>
+      </c>
+      <c r="E198" t="n">
+        <v>23.77</v>
+      </c>
+      <c r="F198" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>RVol: 0.62x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>885.92</v>
+      </c>
+      <c r="D199" t="n">
+        <v>-0.0204</v>
+      </c>
+      <c r="E199" t="n">
+        <v>32</v>
+      </c>
+      <c r="F199" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-10
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M199"/>
+  <dimension ref="A1:M210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12165,6 +12165,655 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>708.6900000000001</v>
+      </c>
+      <c r="D200" t="n">
+        <v>-0.0106</v>
+      </c>
+      <c r="E200" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F200" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>218.36</v>
+      </c>
+      <c r="D201" t="n">
+        <v>-0.0237</v>
+      </c>
+      <c r="E201" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F201" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>326.57</v>
+      </c>
+      <c r="D202" t="n">
+        <v>0.0356</v>
+      </c>
+      <c r="E202" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="F202" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>RVol: 1.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>492.44</v>
+      </c>
+      <c r="D203" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="E203" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="F203" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>RVol: 0.70x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>251.89</v>
+      </c>
+      <c r="D204" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="E204" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="F204" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>644.38</v>
+      </c>
+      <c r="D205" t="n">
+        <v>-0.0142</v>
+      </c>
+      <c r="E205" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="F205" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>RVol: 1.18x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>332.6</v>
+      </c>
+      <c r="D206" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="E206" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F206" t="n">
+        <v>1</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>363.56</v>
+      </c>
+      <c r="D207" t="n">
+        <v>-0.0116</v>
+      </c>
+      <c r="E207" t="n">
+        <v>11.53</v>
+      </c>
+      <c r="F207" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>977.41</v>
+      </c>
+      <c r="D208" t="n">
+        <v>-0.049</v>
+      </c>
+      <c r="E208" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F208" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>460.93</v>
+      </c>
+      <c r="D209" t="n">
+        <v>-0.0443</v>
+      </c>
+      <c r="E209" t="n">
+        <v>14.48</v>
+      </c>
+      <c r="F209" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>RVol: 0.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>862.33</v>
+      </c>
+      <c r="D210" t="n">
+        <v>-0.0266</v>
+      </c>
+      <c r="E210" t="n">
+        <v>32.73</v>
+      </c>
+      <c r="F210" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-12
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M210"/>
+  <dimension ref="A1:M221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12814,6 +12814,655 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>714.88</v>
+      </c>
+      <c r="D211" t="n">
+        <v>0.008699999999999999</v>
+      </c>
+      <c r="E211" t="n">
+        <v>4</v>
+      </c>
+      <c r="F211" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>RVol: 0.84x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>218.29</v>
+      </c>
+      <c r="D212" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="E212" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F212" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>RVol: 0.67x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>332.27</v>
+      </c>
+      <c r="D213" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="E213" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="F213" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>RVol: 1.19x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>495.63</v>
+      </c>
+      <c r="D214" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="E214" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="F214" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>RVol: 0.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>256.78</v>
+      </c>
+      <c r="D215" t="n">
+        <v>0.0194</v>
+      </c>
+      <c r="E215" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="F215" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>648.03</v>
+      </c>
+      <c r="D216" t="n">
+        <v>0.005699999999999999</v>
+      </c>
+      <c r="E216" t="n">
+        <v>18.04</v>
+      </c>
+      <c r="F216" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>338.5</v>
+      </c>
+      <c r="D217" t="n">
+        <v>0.0177</v>
+      </c>
+      <c r="E217" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="F217" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>365.44</v>
+      </c>
+      <c r="D218" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="E218" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="F218" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>975.26</v>
+      </c>
+      <c r="D219" t="n">
+        <v>-0.0022</v>
+      </c>
+      <c r="E219" t="n">
+        <v>26.61</v>
+      </c>
+      <c r="F219" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>447.18</v>
+      </c>
+      <c r="D220" t="n">
+        <v>-0.0298</v>
+      </c>
+      <c r="E220" t="n">
+        <v>29.65</v>
+      </c>
+      <c r="F220" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>830.17</v>
+      </c>
+      <c r="D221" t="n">
+        <v>-0.0373</v>
+      </c>
+      <c r="E221" t="n">
+        <v>53</v>
+      </c>
+      <c r="F221" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-15
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M221"/>
+  <dimension ref="A1:M232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13463,6 +13463,655 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>709.1799999999999</v>
+      </c>
+      <c r="D222" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="E222" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="F222" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>RVol: 1.13x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>210.96</v>
+      </c>
+      <c r="D223" t="n">
+        <v>-0.0336</v>
+      </c>
+      <c r="E223" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="F223" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>RVol: 1.02x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>333.08</v>
+      </c>
+      <c r="D224" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="E224" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="F224" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>505.41</v>
+      </c>
+      <c r="D225" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="E225" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="F225" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>253.54</v>
+      </c>
+      <c r="D226" t="n">
+        <v>-0.0126</v>
+      </c>
+      <c r="E226" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="F226" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>RVol: 1.03x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>665.6</v>
+      </c>
+      <c r="D227" t="n">
+        <v>0.0271</v>
+      </c>
+      <c r="E227" t="n">
+        <v>19.38</v>
+      </c>
+      <c r="F227" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>349.39</v>
+      </c>
+      <c r="D228" t="n">
+        <v>0.0322</v>
+      </c>
+      <c r="E228" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="F228" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>RVol: 1.53x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>358.97</v>
+      </c>
+      <c r="D229" t="n">
+        <v>-0.0177</v>
+      </c>
+      <c r="E229" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F229" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>924.03</v>
+      </c>
+      <c r="D230" t="n">
+        <v>-0.0525</v>
+      </c>
+      <c r="E230" t="n">
+        <v>29.61</v>
+      </c>
+      <c r="F230" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>RVol: 1.03x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>426.94</v>
+      </c>
+      <c r="D231" t="n">
+        <v>-0.0453</v>
+      </c>
+      <c r="E231" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="F231" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>805.55</v>
+      </c>
+      <c r="D232" t="n">
+        <v>-0.0297</v>
+      </c>
+      <c r="E232" t="n">
+        <v>52.86</v>
+      </c>
+      <c r="F232" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>RVol: 1.15x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-16
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M232"/>
+  <dimension ref="A1:M243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14112,6 +14112,655 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>704.54</v>
+      </c>
+      <c r="D233" t="n">
+        <v>-0.006500000000000001</v>
+      </c>
+      <c r="E233" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="F233" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>212.17</v>
+      </c>
+      <c r="D234" t="n">
+        <v>0.005699999999999999</v>
+      </c>
+      <c r="E234" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>RVol: 0.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>331.34</v>
+      </c>
+      <c r="D235" t="n">
+        <v>-0.0052</v>
+      </c>
+      <c r="E235" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F235" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>497.12</v>
+      </c>
+      <c r="D236" t="n">
+        <v>-0.0164</v>
+      </c>
+      <c r="E236" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F236" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>248.42</v>
+      </c>
+      <c r="D237" t="n">
+        <v>-0.0202</v>
+      </c>
+      <c r="E237" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="F237" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>670.24</v>
+      </c>
+      <c r="D238" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="E238" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="F238" t="n">
+        <v>1</v>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>344.98</v>
+      </c>
+      <c r="D239" t="n">
+        <v>-0.0126</v>
+      </c>
+      <c r="E239" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="F239" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>356.58</v>
+      </c>
+      <c r="D240" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="E240" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="F240" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>927.6</v>
+      </c>
+      <c r="D241" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="E241" t="n">
+        <v>24.81</v>
+      </c>
+      <c r="F241" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>411.96</v>
+      </c>
+      <c r="D242" t="n">
+        <v>-0.0351</v>
+      </c>
+      <c r="E242" t="n">
+        <v>23.13</v>
+      </c>
+      <c r="F242" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>RVol: 1.27x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>771.8099999999999</v>
+      </c>
+      <c r="D243" t="n">
+        <v>-0.04190000000000001</v>
+      </c>
+      <c r="E243" t="n">
+        <v>43.63</v>
+      </c>
+      <c r="F243" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>RVol: 1.13x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-17
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M243"/>
+  <dimension ref="A1:M254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14761,6 +14761,655 @@
         </is>
       </c>
     </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>704.72</v>
+      </c>
+      <c r="D244" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="E244" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="F244" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>RVol: 1.12x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>213.9</v>
+      </c>
+      <c r="D245" t="n">
+        <v>0.008199999999999999</v>
+      </c>
+      <c r="E245" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="F245" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>332.41</v>
+      </c>
+      <c r="D246" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="E246" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="F246" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>490.3</v>
+      </c>
+      <c r="D247" t="n">
+        <v>-0.0137</v>
+      </c>
+      <c r="E247" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="F247" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>245.96</v>
+      </c>
+      <c r="D248" t="n">
+        <v>-0.009899999999999999</v>
+      </c>
+      <c r="E248" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="F248" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>RVol: 1.03x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>673.3099999999999</v>
+      </c>
+      <c r="D249" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="E249" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="F249" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>342.87</v>
+      </c>
+      <c r="D250" t="n">
+        <v>-0.0061</v>
+      </c>
+      <c r="E250" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="F250" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>358.08</v>
+      </c>
+      <c r="D251" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="E251" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>926.55</v>
+      </c>
+      <c r="D252" t="n">
+        <v>-0.0011</v>
+      </c>
+      <c r="E252" t="n">
+        <v>23.56</v>
+      </c>
+      <c r="F252" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>416.97</v>
+      </c>
+      <c r="D253" t="n">
+        <v>0.0122</v>
+      </c>
+      <c r="E253" t="n">
+        <v>13.54</v>
+      </c>
+      <c r="F253" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>RVol: 1.22x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>783.1799999999999</v>
+      </c>
+      <c r="D254" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="E254" t="n">
+        <v>26.87</v>
+      </c>
+      <c r="F254" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-18
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M254"/>
+  <dimension ref="A1:M265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15410,6 +15410,655 @@
         </is>
       </c>
     </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>716.92</v>
+      </c>
+      <c r="D255" t="n">
+        <v>0.0173</v>
+      </c>
+      <c r="E255" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="F255" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>RVol: 1.18x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>219.34</v>
+      </c>
+      <c r="D256" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="E256" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="F256" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>RVol: 0.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>337</v>
+      </c>
+      <c r="D257" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="E257" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="F257" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>RVol: 0.86x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>497.75</v>
+      </c>
+      <c r="D258" t="n">
+        <v>0.0152</v>
+      </c>
+      <c r="E258" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="F258" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>251.19</v>
+      </c>
+      <c r="D259" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="E259" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F259" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>682.3099999999999</v>
+      </c>
+      <c r="D260" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="E260" t="n">
+        <v>16.15</v>
+      </c>
+      <c r="F260" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>347.33</v>
+      </c>
+      <c r="D261" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="E261" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="F261" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>366.2</v>
+      </c>
+      <c r="D262" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="E262" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="F262" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>RVol: 0.96x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>977.5</v>
+      </c>
+      <c r="D263" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="E263" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>423.87</v>
+      </c>
+      <c r="D264" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="E264" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="F264" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>RVol: 1.15x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>803.13</v>
+      </c>
+      <c r="D265" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="E265" t="n">
+        <v>33.67</v>
+      </c>
+      <c r="F265" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>RVol: 1.39x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-19
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M265"/>
+  <dimension ref="A1:M276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16059,6 +16059,655 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>721.45</v>
+      </c>
+      <c r="D266" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="E266" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F266" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>RVol: 1.55x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>222.27</v>
+      </c>
+      <c r="D267" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="E267" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F267" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>RVol: 1.44x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>336.13</v>
+      </c>
+      <c r="D268" t="n">
+        <v>-0.0026</v>
+      </c>
+      <c r="E268" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="F268" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>RVol: 2.09x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>493.78</v>
+      </c>
+      <c r="D269" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="E269" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="F269" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>RVol: 1.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>253.71</v>
+      </c>
+      <c r="D270" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E270" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F270" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>RVol: 1.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>665.75</v>
+      </c>
+      <c r="D271" t="n">
+        <v>-0.0243</v>
+      </c>
+      <c r="E271" t="n">
+        <v>29.35</v>
+      </c>
+      <c r="F271" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>RVol: 1.52x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>349.54</v>
+      </c>
+      <c r="D272" t="n">
+        <v>0.0064</v>
+      </c>
+      <c r="E272" t="n">
+        <v>11</v>
+      </c>
+      <c r="F272" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>RVol: 1.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>364.27</v>
+      </c>
+      <c r="D273" t="n">
+        <v>-0.0053</v>
+      </c>
+      <c r="E273" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="F273" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>RVol: 1.31x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>1015.8</v>
+      </c>
+      <c r="D274" t="n">
+        <v>0.0392</v>
+      </c>
+      <c r="E274" t="n">
+        <v>38.61</v>
+      </c>
+      <c r="F274" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>RVol: 1.44x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>441.36</v>
+      </c>
+      <c r="D275" t="n">
+        <v>0.0413</v>
+      </c>
+      <c r="E275" t="n">
+        <v>24.31</v>
+      </c>
+      <c r="F275" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>RVol: 2.31x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>858.79</v>
+      </c>
+      <c r="D276" t="n">
+        <v>0.0693</v>
+      </c>
+      <c r="E276" t="n">
+        <v>64.97</v>
+      </c>
+      <c r="F276" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>RVol: 2.03x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-22
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M276"/>
+  <dimension ref="A1:M287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16708,6 +16708,655 @@
         </is>
       </c>
     </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>741.47</v>
+      </c>
+      <c r="D277" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="E277" t="n">
+        <v>15.41</v>
+      </c>
+      <c r="F277" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>RVol: 1.47x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>227.38</v>
+      </c>
+      <c r="D278" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="E278" t="n">
+        <v>6.94</v>
+      </c>
+      <c r="F278" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>338.98</v>
+      </c>
+      <c r="D279" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="E279" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="F279" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>501.61</v>
+      </c>
+      <c r="D280" t="n">
+        <v>0.0159</v>
+      </c>
+      <c r="E280" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="F280" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>RVol: 1.24x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>258.45</v>
+      </c>
+      <c r="D281" t="n">
+        <v>0.0187</v>
+      </c>
+      <c r="E281" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="F281" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>RVol: 1.24x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>741.24</v>
+      </c>
+      <c r="D282" t="n">
+        <v>0.1134</v>
+      </c>
+      <c r="E282" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="F282" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>RVol: 2.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>354.97</v>
+      </c>
+      <c r="D283" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="E283" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="F283" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>375.3</v>
+      </c>
+      <c r="D284" t="n">
+        <v>0.0303</v>
+      </c>
+      <c r="E284" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="F284" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>1043.96</v>
+      </c>
+      <c r="D285" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="E285" t="n">
+        <v>33.81</v>
+      </c>
+      <c r="F285" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>RVol: 1.09x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>448.17</v>
+      </c>
+      <c r="D286" t="n">
+        <v>0.0154</v>
+      </c>
+      <c r="E286" t="n">
+        <v>23.29</v>
+      </c>
+      <c r="F286" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>RVol: 1.19x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>877.3200000000001</v>
+      </c>
+      <c r="D287" t="n">
+        <v>0.0216</v>
+      </c>
+      <c r="E287" t="n">
+        <v>52.86</v>
+      </c>
+      <c r="F287" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>RVol: 1.16x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-23
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M287"/>
+  <dimension ref="A1:M298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17357,6 +17357,655 @@
         </is>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>747.46</v>
+      </c>
+      <c r="D288" t="n">
+        <v>0.008100000000000001</v>
+      </c>
+      <c r="E288" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="F288" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>RVol: 1.22x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>228.87</v>
+      </c>
+      <c r="D289" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="E289" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>RVol: 0.69x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>339.75</v>
+      </c>
+      <c r="D290" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="E290" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="F290" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>498</v>
+      </c>
+      <c r="D291" t="n">
+        <v>-0.0072</v>
+      </c>
+      <c r="E291" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>254.98</v>
+      </c>
+      <c r="D292" t="n">
+        <v>-0.0134</v>
+      </c>
+      <c r="E292" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="F292" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>RVol: 1.24x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>736.6</v>
+      </c>
+      <c r="D293" t="n">
+        <v>-0.0063</v>
+      </c>
+      <c r="E293" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="F293" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>RVol: 1.36x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>351.16</v>
+      </c>
+      <c r="D294" t="n">
+        <v>-0.0107</v>
+      </c>
+      <c r="E294" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="F294" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>RVol: 1.13x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>378.9</v>
+      </c>
+      <c r="D295" t="n">
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="E295" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>RVol: 0.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>1096.16</v>
+      </c>
+      <c r="D296" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E296" t="n">
+        <v>67.23</v>
+      </c>
+      <c r="F296" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>RVol: 1.14x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>464.6</v>
+      </c>
+      <c r="D297" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="E297" t="n">
+        <v>36.54</v>
+      </c>
+      <c r="F297" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>RVol: 1.31x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>919.84</v>
+      </c>
+      <c r="D298" t="n">
+        <v>0.04849999999999999</v>
+      </c>
+      <c r="E298" t="n">
+        <v>80.55</v>
+      </c>
+      <c r="F298" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>RVol: 1.43x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-24
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M298"/>
+  <dimension ref="A1:M309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18006,6 +18006,655 @@
         </is>
       </c>
     </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>741.21</v>
+      </c>
+      <c r="D299" t="n">
+        <v>-0.008399999999999999</v>
+      </c>
+      <c r="E299" t="n">
+        <v>8.94</v>
+      </c>
+      <c r="F299" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>RVol: 1.01x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>225.51</v>
+      </c>
+      <c r="D300" t="n">
+        <v>-0.0147</v>
+      </c>
+      <c r="E300" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>RVol: 0.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>337.02</v>
+      </c>
+      <c r="D301" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="E301" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>500.59</v>
+      </c>
+      <c r="D302" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="E302" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="F302" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>249.27</v>
+      </c>
+      <c r="D303" t="n">
+        <v>-0.0224</v>
+      </c>
+      <c r="E303" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="F303" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>RVol: 1.29x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>744.1</v>
+      </c>
+      <c r="D304" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="E304" t="n">
+        <v>24.39</v>
+      </c>
+      <c r="F304" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>RVol: 1.42x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>337.83</v>
+      </c>
+      <c r="D305" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="E305" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="F305" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>RVol: 1.35x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>380.12</v>
+      </c>
+      <c r="D306" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="E306" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>1071.88</v>
+      </c>
+      <c r="D307" t="n">
+        <v>-0.0222</v>
+      </c>
+      <c r="E307" t="n">
+        <v>41.25</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>473.69</v>
+      </c>
+      <c r="D308" t="n">
+        <v>0.0196</v>
+      </c>
+      <c r="E308" t="n">
+        <v>30.64</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>923.86</v>
+      </c>
+      <c r="D309" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="E309" t="n">
+        <v>42</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-25
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M309"/>
+  <dimension ref="A1:M320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18655,6 +18655,655 @@
         </is>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>741.1</v>
+      </c>
+      <c r="D310" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="E310" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>224.58</v>
+      </c>
+      <c r="D311" t="n">
+        <v>-0.004099999999999999</v>
+      </c>
+      <c r="E311" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>RVol: 0.58x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>335.92</v>
+      </c>
+      <c r="D312" t="n">
+        <v>-0.0033</v>
+      </c>
+      <c r="E312" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>RVol: 0.56x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>497.93</v>
+      </c>
+      <c r="D313" t="n">
+        <v>-0.0053</v>
+      </c>
+      <c r="E313" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>249.38</v>
+      </c>
+      <c r="D314" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="E314" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>777.59</v>
+      </c>
+      <c r="D315" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="E315" t="n">
+        <v>36.81</v>
+      </c>
+      <c r="F315" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>RVol: 1.55x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>342.36</v>
+      </c>
+      <c r="D316" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="E316" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>377.94</v>
+      </c>
+      <c r="D317" t="n">
+        <v>-0.005699999999999999</v>
+      </c>
+      <c r="E317" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>RVol: 0.66x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>1080.53</v>
+      </c>
+      <c r="D318" t="n">
+        <v>0.008100000000000001</v>
+      </c>
+      <c r="E318" t="n">
+        <v>37.04</v>
+      </c>
+      <c r="F318" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>450.31</v>
+      </c>
+      <c r="D319" t="n">
+        <v>-0.04940000000000001</v>
+      </c>
+      <c r="E319" t="n">
+        <v>18.79</v>
+      </c>
+      <c r="F319" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>905.92</v>
+      </c>
+      <c r="D320" t="n">
+        <v>-0.0194</v>
+      </c>
+      <c r="E320" t="n">
+        <v>27.21</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-26
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M320"/>
+  <dimension ref="A1:M331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19304,6 +19304,655 @@
         </is>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>744.5</v>
+      </c>
+      <c r="D321" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="E321" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>225.07</v>
+      </c>
+      <c r="D322" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="E322" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>RVol: 0.69x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>341.07</v>
+      </c>
+      <c r="D323" t="n">
+        <v>0.0153</v>
+      </c>
+      <c r="E323" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>RVol: 0.69x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>516.17</v>
+      </c>
+      <c r="D324" t="n">
+        <v>0.0366</v>
+      </c>
+      <c r="E324" t="n">
+        <v>22.15</v>
+      </c>
+      <c r="F324" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>RVol: 1.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>249.67</v>
+      </c>
+      <c r="D325" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="E325" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F325" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>751.66</v>
+      </c>
+      <c r="D326" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="E326" t="n">
+        <v>23.03</v>
+      </c>
+      <c r="F326" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>RVol: 1.14x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>343.92</v>
+      </c>
+      <c r="D327" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="E327" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="F327" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>372.11</v>
+      </c>
+      <c r="D328" t="n">
+        <v>-0.0154</v>
+      </c>
+      <c r="E328" t="n">
+        <v>19.16</v>
+      </c>
+      <c r="F328" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>RVol: 1.15x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>1082.28</v>
+      </c>
+      <c r="D329" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="E329" t="n">
+        <v>35.72</v>
+      </c>
+      <c r="F329" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>456.81</v>
+      </c>
+      <c r="D330" t="n">
+        <v>0.0144</v>
+      </c>
+      <c r="E330" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="F330" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
+        <v>916.83</v>
+      </c>
+      <c r="D331" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="E331" t="n">
+        <v>20.83</v>
+      </c>
+      <c r="F331" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-29
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M331"/>
+  <dimension ref="A1:M342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19953,6 +19953,655 @@
         </is>
       </c>
     </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>736.53</v>
+      </c>
+      <c r="D332" t="n">
+        <v>-0.0107</v>
+      </c>
+      <c r="E332" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F332" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>RVol: 1.26x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>228.86</v>
+      </c>
+      <c r="D333" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="E333" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="F333" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>RVol: 1.23x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>338.4</v>
+      </c>
+      <c r="D334" t="n">
+        <v>-0.007800000000000001</v>
+      </c>
+      <c r="E334" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="F334" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>509.22</v>
+      </c>
+      <c r="D335" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="E335" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="F335" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>246.15</v>
+      </c>
+      <c r="D336" t="n">
+        <v>-0.0141</v>
+      </c>
+      <c r="E336" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="F336" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>715.62</v>
+      </c>
+      <c r="D337" t="n">
+        <v>-0.0479</v>
+      </c>
+      <c r="E337" t="n">
+        <v>37.39</v>
+      </c>
+      <c r="F337" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>RVol: 1.22x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>342.75</v>
+      </c>
+      <c r="D338" t="n">
+        <v>-0.0034</v>
+      </c>
+      <c r="E338" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="F338" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
+        <v>357.45</v>
+      </c>
+      <c r="D339" t="n">
+        <v>-0.0394</v>
+      </c>
+      <c r="E339" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="F339" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>1053.98</v>
+      </c>
+      <c r="D340" t="n">
+        <v>-0.0261</v>
+      </c>
+      <c r="E340" t="n">
+        <v>52.81</v>
+      </c>
+      <c r="F340" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>453.23</v>
+      </c>
+      <c r="D341" t="n">
+        <v>-0.007800000000000001</v>
+      </c>
+      <c r="E341" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="F341" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>RVol: 1.15x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C342" t="n">
+        <v>921.51</v>
+      </c>
+      <c r="D342" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="E342" t="n">
+        <v>62.49</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>RVol: 0.91x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-30
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M342"/>
+  <dimension ref="A1:M353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20602,6 +20602,655 @@
         </is>
       </c>
     </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C343" t="n">
+        <v>737.9299999999999</v>
+      </c>
+      <c r="D343" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="E343" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="F343" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>RVol: 0.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C344" t="n">
+        <v>227.21</v>
+      </c>
+      <c r="D344" t="n">
+        <v>-0.0072</v>
+      </c>
+      <c r="E344" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="F344" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K344" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>RVol: 0.86x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C345" t="n">
+        <v>329.4</v>
+      </c>
+      <c r="D345" t="n">
+        <v>-0.0266</v>
+      </c>
+      <c r="E345" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="F345" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C346" t="n">
+        <v>508.96</v>
+      </c>
+      <c r="D346" t="n">
+        <v>-0.0005</v>
+      </c>
+      <c r="E346" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="F346" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C347" t="n">
+        <v>246.67</v>
+      </c>
+      <c r="D347" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="E347" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F347" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>RVol: 0.91x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C348" t="n">
+        <v>738.79</v>
+      </c>
+      <c r="D348" t="n">
+        <v>0.03240000000000001</v>
+      </c>
+      <c r="E348" t="n">
+        <v>25.35</v>
+      </c>
+      <c r="F348" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K348" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>RVol: 0.98x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C349" t="n">
+        <v>340.92</v>
+      </c>
+      <c r="D349" t="n">
+        <v>-0.0053</v>
+      </c>
+      <c r="E349" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="F349" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C350" t="n">
+        <v>352.84</v>
+      </c>
+      <c r="D350" t="n">
+        <v>-0.0129</v>
+      </c>
+      <c r="E350" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="F350" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C351" t="n">
+        <v>1065.08</v>
+      </c>
+      <c r="D351" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="E351" t="n">
+        <v>24.96</v>
+      </c>
+      <c r="F351" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C352" t="n">
+        <v>453.48</v>
+      </c>
+      <c r="D352" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="E352" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C353" t="n">
+        <v>913.45</v>
+      </c>
+      <c r="D353" t="n">
+        <v>-0.008699999999999999</v>
+      </c>
+      <c r="E353" t="n">
+        <v>44.33</v>
+      </c>
+      <c r="F353" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>RVol: 0.67x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-01
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M353"/>
+  <dimension ref="A1:M364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21251,6 +21251,655 @@
         </is>
       </c>
     </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C354" t="n">
+        <v>739.77</v>
+      </c>
+      <c r="D354" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="E354" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="F354" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>228.38</v>
+      </c>
+      <c r="D355" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="E355" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F355" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>RVol: 1.05x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C356" t="n">
+        <v>333.02</v>
+      </c>
+      <c r="D356" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="E356" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F356" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>RVol: 1.16x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>512.9</v>
+      </c>
+      <c r="D357" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="E357" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F357" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>RVol: 1.28x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>249.15</v>
+      </c>
+      <c r="D358" t="n">
+        <v>0.0101</v>
+      </c>
+      <c r="E358" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="F358" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>RVol: 1.22x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>725.1799999999999</v>
+      </c>
+      <c r="D359" t="n">
+        <v>-0.0184</v>
+      </c>
+      <c r="E359" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="F359" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>344.08</v>
+      </c>
+      <c r="D360" t="n">
+        <v>0.009300000000000001</v>
+      </c>
+      <c r="E360" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="F360" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>RVol: 1.39x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>354.81</v>
+      </c>
+      <c r="D361" t="n">
+        <v>0.005600000000000001</v>
+      </c>
+      <c r="E361" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="F361" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>1065.11</v>
+      </c>
+      <c r="D362" t="n">
+        <v>0</v>
+      </c>
+      <c r="E362" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="F362" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>RVol: 1.25x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>454.46</v>
+      </c>
+      <c r="D363" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="E363" t="n">
+        <v>17.65</v>
+      </c>
+      <c r="F363" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>RVol: 1.04x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>922.34</v>
+      </c>
+      <c r="D364" t="n">
+        <v>0.0097</v>
+      </c>
+      <c r="E364" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="F364" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-02
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M364"/>
+  <dimension ref="A1:M375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21900,6 +21900,655 @@
         </is>
       </c>
     </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>742.03</v>
+      </c>
+      <c r="D365" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="E365" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="F365" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>230.86</v>
+      </c>
+      <c r="D366" t="n">
+        <v>0.0109</v>
+      </c>
+      <c r="E366" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="F366" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>330.32</v>
+      </c>
+      <c r="D367" t="n">
+        <v>-0.008100000000000001</v>
+      </c>
+      <c r="E367" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>RVol: 0.86x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>512.8</v>
+      </c>
+      <c r="D368" t="n">
+        <v>-0.0002</v>
+      </c>
+      <c r="E368" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="F368" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>248.23</v>
+      </c>
+      <c r="D369" t="n">
+        <v>-0.0037</v>
+      </c>
+      <c r="E369" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="F369" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>725.9299999999999</v>
+      </c>
+      <c r="D370" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E370" t="n">
+        <v>14.37</v>
+      </c>
+      <c r="F370" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>RVol: 0.51x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>338.24</v>
+      </c>
+      <c r="D371" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="E371" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="F371" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>RVol: 1.25x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>354.11</v>
+      </c>
+      <c r="D372" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="E372" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F372" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>1097.39</v>
+      </c>
+      <c r="D373" t="n">
+        <v>0.0303</v>
+      </c>
+      <c r="E373" t="n">
+        <v>76</v>
+      </c>
+      <c r="F373" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>RVol: 1.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>462.56</v>
+      </c>
+      <c r="D374" t="n">
+        <v>0.0178</v>
+      </c>
+      <c r="E374" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F374" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>945.5700000000001</v>
+      </c>
+      <c r="D375" t="n">
+        <v>0.0252</v>
+      </c>
+      <c r="E375" t="n">
+        <v>52.62</v>
+      </c>
+      <c r="F375" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>RVol: 0.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-03
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M375"/>
+  <dimension ref="A1:M386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22549,6 +22549,655 @@
         </is>
       </c>
     </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>749.58</v>
+      </c>
+      <c r="D376" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="E376" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="F376" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>RVol: 1.01x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>233.95</v>
+      </c>
+      <c r="D377" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="E377" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="F377" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>RVol: 1.22x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>333.69</v>
+      </c>
+      <c r="D378" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="E378" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="F378" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>517.53</v>
+      </c>
+      <c r="D379" t="n">
+        <v>0.0092</v>
+      </c>
+      <c r="E379" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="F379" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>251.52</v>
+      </c>
+      <c r="D380" t="n">
+        <v>0.0133</v>
+      </c>
+      <c r="E380" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="F380" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>728.08</v>
+      </c>
+      <c r="D381" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="E381" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="F381" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>RVol: 0.54x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>343.5</v>
+      </c>
+      <c r="D382" t="n">
+        <v>0.0156</v>
+      </c>
+      <c r="E382" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="F382" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>370.59</v>
+      </c>
+      <c r="D383" t="n">
+        <v>0.04650000000000001</v>
+      </c>
+      <c r="E383" t="n">
+        <v>15.19</v>
+      </c>
+      <c r="F383" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>RVol: 1.40x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>1074.89</v>
+      </c>
+      <c r="D384" t="n">
+        <v>-0.0205</v>
+      </c>
+      <c r="E384" t="n">
+        <v>35.99</v>
+      </c>
+      <c r="F384" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>RVol: 1.01x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>415.29</v>
+      </c>
+      <c r="D385" t="n">
+        <v>-0.1022</v>
+      </c>
+      <c r="E385" t="n">
+        <v>31.14</v>
+      </c>
+      <c r="F385" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>RVol: 3.63x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>848.99</v>
+      </c>
+      <c r="D386" t="n">
+        <v>-0.1021</v>
+      </c>
+      <c r="E386" t="n">
+        <v>60.54</v>
+      </c>
+      <c r="F386" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>RVol: 3.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-06
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M386"/>
+  <dimension ref="A1:M397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23198,6 +23198,655 @@
         </is>
       </c>
     </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>756.2</v>
+      </c>
+      <c r="D387" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="E387" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="F387" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>RVol: 0.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C388" t="n">
+        <v>238.9</v>
+      </c>
+      <c r="D388" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="E388" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="F388" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>RVol: 1.16x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C389" t="n">
+        <v>332.89</v>
+      </c>
+      <c r="D389" t="n">
+        <v>-0.0024</v>
+      </c>
+      <c r="E389" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="F389" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C390" t="n">
+        <v>525.1799999999999</v>
+      </c>
+      <c r="D390" t="n">
+        <v>0.0148</v>
+      </c>
+      <c r="E390" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="F390" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>RVol: 1.25x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C391" t="n">
+        <v>251.4</v>
+      </c>
+      <c r="D391" t="n">
+        <v>-0.0005</v>
+      </c>
+      <c r="E391" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="F391" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>RVol: 1.12x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C392" t="n">
+        <v>741.9</v>
+      </c>
+      <c r="D392" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="E392" t="n">
+        <v>19.58</v>
+      </c>
+      <c r="F392" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>RVol: 0.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C393" t="n">
+        <v>346.47</v>
+      </c>
+      <c r="D393" t="n">
+        <v>0.0086</v>
+      </c>
+      <c r="E393" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="F393" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C394" t="n">
+        <v>378.73</v>
+      </c>
+      <c r="D394" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="E394" t="n">
+        <v>16.68</v>
+      </c>
+      <c r="F394" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>1063.96</v>
+      </c>
+      <c r="D395" t="n">
+        <v>-0.0102</v>
+      </c>
+      <c r="E395" t="n">
+        <v>19.32</v>
+      </c>
+      <c r="F395" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>RVol: 0.69x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>441.64</v>
+      </c>
+      <c r="D396" t="n">
+        <v>0.0634</v>
+      </c>
+      <c r="E396" t="n">
+        <v>18.27</v>
+      </c>
+      <c r="F396" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>RVol: 1.46x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>887.09</v>
+      </c>
+      <c r="D397" t="n">
+        <v>0.0449</v>
+      </c>
+      <c r="E397" t="n">
+        <v>28</v>
+      </c>
+      <c r="F397" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>RVol: 1.30x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-07
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M397"/>
+  <dimension ref="A1:M408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23847,6 +23847,655 @@
         </is>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>759.66</v>
+      </c>
+      <c r="D398" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="E398" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="F398" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C399" t="n">
+        <v>239.24</v>
+      </c>
+      <c r="D399" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="E399" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="F399" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>333.63</v>
+      </c>
+      <c r="D400" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="E400" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="F400" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>RVol: 0.70x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>529.3</v>
+      </c>
+      <c r="D401" t="n">
+        <v>0.007800000000000001</v>
+      </c>
+      <c r="E401" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="F401" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>256.29</v>
+      </c>
+      <c r="D402" t="n">
+        <v>0.0195</v>
+      </c>
+      <c r="E402" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="F402" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>RVol: 0.96x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C403" t="n">
+        <v>738.88</v>
+      </c>
+      <c r="D403" t="n">
+        <v>-0.004099999999999999</v>
+      </c>
+      <c r="E403" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="F403" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>RVol: 0.51x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C404" t="n">
+        <v>347.68</v>
+      </c>
+      <c r="D404" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="E404" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="F404" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>RVol: 0.67x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>380.68</v>
+      </c>
+      <c r="D405" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="E405" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="F405" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>1045.56</v>
+      </c>
+      <c r="D406" t="n">
+        <v>-0.0173</v>
+      </c>
+      <c r="E406" t="n">
+        <v>29.05</v>
+      </c>
+      <c r="F406" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>411.04</v>
+      </c>
+      <c r="D407" t="n">
+        <v>-0.0693</v>
+      </c>
+      <c r="E407" t="n">
+        <v>23.52</v>
+      </c>
+      <c r="F407" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>RVol: 1.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>805.63</v>
+      </c>
+      <c r="D408" t="n">
+        <v>-0.09179999999999999</v>
+      </c>
+      <c r="E408" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="F408" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>RVol: 1.62x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-08
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M408"/>
+  <dimension ref="A1:M419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24496,6 +24496,655 @@
         </is>
       </c>
     </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>757.73</v>
+      </c>
+      <c r="D409" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="E409" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="F409" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>237.47</v>
+      </c>
+      <c r="D410" t="n">
+        <v>-0.0074</v>
+      </c>
+      <c r="E410" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F410" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C411" t="n">
+        <v>336.67</v>
+      </c>
+      <c r="D411" t="n">
+        <v>0.0091</v>
+      </c>
+      <c r="E411" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="F411" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>529.76</v>
+      </c>
+      <c r="D412" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="E412" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="F412" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>259.92</v>
+      </c>
+      <c r="D413" t="n">
+        <v>0.0142</v>
+      </c>
+      <c r="E413" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="F413" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>721.3099999999999</v>
+      </c>
+      <c r="D414" t="n">
+        <v>-0.0238</v>
+      </c>
+      <c r="E414" t="n">
+        <v>18.14</v>
+      </c>
+      <c r="F414" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>RVol: 0.55x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>350.5</v>
+      </c>
+      <c r="D415" t="n">
+        <v>0.008100000000000001</v>
+      </c>
+      <c r="E415" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="F415" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>377.81</v>
+      </c>
+      <c r="D416" t="n">
+        <v>-0.0075</v>
+      </c>
+      <c r="E416" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="F416" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>RVol: 0.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>1088</v>
+      </c>
+      <c r="D417" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="E417" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="F417" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>RVol: 1.19x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>405.42</v>
+      </c>
+      <c r="D418" t="n">
+        <v>-0.0137</v>
+      </c>
+      <c r="E418" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="F418" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>807.5700000000001</v>
+      </c>
+      <c r="D419" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="E419" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="F419" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-09
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M419"/>
+  <dimension ref="A1:M430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25145,6 +25145,655 @@
         </is>
       </c>
     </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>747.58</v>
+      </c>
+      <c r="D420" t="n">
+        <v>-0.0134</v>
+      </c>
+      <c r="E420" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="F420" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>RVol: 1.49x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>230.48</v>
+      </c>
+      <c r="D421" t="n">
+        <v>-0.0294</v>
+      </c>
+      <c r="E421" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="F421" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>RVol: 1.09x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C422" t="n">
+        <v>340.42</v>
+      </c>
+      <c r="D422" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="E422" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="F422" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>522.61</v>
+      </c>
+      <c r="D423" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="E423" t="n">
+        <v>14.72</v>
+      </c>
+      <c r="F423" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>254.06</v>
+      </c>
+      <c r="D424" t="n">
+        <v>-0.0225</v>
+      </c>
+      <c r="E424" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="F424" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>720.89</v>
+      </c>
+      <c r="D425" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="E425" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="F425" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>348.29</v>
+      </c>
+      <c r="D426" t="n">
+        <v>-0.0063</v>
+      </c>
+      <c r="E426" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="F426" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C427" t="n">
+        <v>375</v>
+      </c>
+      <c r="D427" t="n">
+        <v>-0.0074</v>
+      </c>
+      <c r="E427" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="F427" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C428" t="n">
+        <v>1035.84</v>
+      </c>
+      <c r="D428" t="n">
+        <v>-0.0479</v>
+      </c>
+      <c r="E428" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="F428" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>RVol: 1.17x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C429" t="n">
+        <v>393.31</v>
+      </c>
+      <c r="D429" t="n">
+        <v>-0.0299</v>
+      </c>
+      <c r="E429" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="F429" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>RVol: 1.01x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C430" t="n">
+        <v>774.8200000000001</v>
+      </c>
+      <c r="D430" t="n">
+        <v>-0.0405</v>
+      </c>
+      <c r="E430" t="n">
+        <v>31.89</v>
+      </c>
+      <c r="F430" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-10
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M430"/>
+  <dimension ref="A1:M441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25794,6 +25794,655 @@
         </is>
       </c>
     </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C431" t="n">
+        <v>751.27</v>
+      </c>
+      <c r="D431" t="n">
+        <v>0.0049</v>
+      </c>
+      <c r="E431" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F431" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>RVol: 0.60x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C432" t="n">
+        <v>229.28</v>
+      </c>
+      <c r="D432" t="n">
+        <v>-0.0052</v>
+      </c>
+      <c r="E432" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="F432" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C433" t="n">
+        <v>336.64</v>
+      </c>
+      <c r="D433" t="n">
+        <v>-0.0111</v>
+      </c>
+      <c r="E433" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="F433" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C434" t="n">
+        <v>535.0700000000001</v>
+      </c>
+      <c r="D434" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="E434" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="F434" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C435" t="n">
+        <v>262.43</v>
+      </c>
+      <c r="D435" t="n">
+        <v>0.0329</v>
+      </c>
+      <c r="E435" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F435" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>RVol: 0.91x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C436" t="n">
+        <v>718.67</v>
+      </c>
+      <c r="D436" t="n">
+        <v>-0.0031</v>
+      </c>
+      <c r="E436" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="F436" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>RVol: 0.58x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C437" t="n">
+        <v>351.66</v>
+      </c>
+      <c r="D437" t="n">
+        <v>0.0097</v>
+      </c>
+      <c r="E437" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F437" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>RVol: 0.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C438" t="n">
+        <v>382.7</v>
+      </c>
+      <c r="D438" t="n">
+        <v>0.0205</v>
+      </c>
+      <c r="E438" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="F438" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C439" t="n">
+        <v>1029</v>
+      </c>
+      <c r="D439" t="n">
+        <v>-0.0066</v>
+      </c>
+      <c r="E439" t="n">
+        <v>37.17</v>
+      </c>
+      <c r="F439" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C440" t="n">
+        <v>397.28</v>
+      </c>
+      <c r="D440" t="n">
+        <v>0.0101</v>
+      </c>
+      <c r="E440" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="F440" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C441" t="n">
+        <v>783</v>
+      </c>
+      <c r="D441" t="n">
+        <v>0.0106</v>
+      </c>
+      <c r="E441" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F441" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-13
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M441"/>
+  <dimension ref="A1:M452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26443,6 +26443,655 @@
         </is>
       </c>
     </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C442" t="n">
+        <v>746.04</v>
+      </c>
+      <c r="D442" t="n">
+        <v>-0.006999999999999999</v>
+      </c>
+      <c r="E442" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="F442" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C443" t="n">
+        <v>226.32</v>
+      </c>
+      <c r="D443" t="n">
+        <v>-0.0129</v>
+      </c>
+      <c r="E443" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F443" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>RVol: 0.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C444" t="n">
+        <v>340.97</v>
+      </c>
+      <c r="D444" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="E444" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="F444" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>RVol: 0.69x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C445" t="n">
+        <v>541.15</v>
+      </c>
+      <c r="D445" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="E445" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="F445" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C446" t="n">
+        <v>259.53</v>
+      </c>
+      <c r="D446" t="n">
+        <v>-0.0111</v>
+      </c>
+      <c r="E446" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="F446" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C447" t="n">
+        <v>742.96</v>
+      </c>
+      <c r="D447" t="n">
+        <v>0.0338</v>
+      </c>
+      <c r="E447" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="F447" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>RVol: 1.15x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C448" t="n">
+        <v>352.72</v>
+      </c>
+      <c r="D448" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="E448" t="n">
+        <v>6</v>
+      </c>
+      <c r="F448" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C449" t="n">
+        <v>378.03</v>
+      </c>
+      <c r="D449" t="n">
+        <v>-0.0122</v>
+      </c>
+      <c r="E449" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="F449" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>RVol: 0.56x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C450" t="n">
+        <v>989.04</v>
+      </c>
+      <c r="D450" t="n">
+        <v>-0.0388</v>
+      </c>
+      <c r="E450" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="F450" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C451" t="n">
+        <v>386.94</v>
+      </c>
+      <c r="D451" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="E451" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="F451" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>RVol: 0.61x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C452" t="n">
+        <v>753.25</v>
+      </c>
+      <c r="D452" t="n">
+        <v>-0.038</v>
+      </c>
+      <c r="E452" t="n">
+        <v>19.32</v>
+      </c>
+      <c r="F452" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-14
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M452"/>
+  <dimension ref="A1:M463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27092,6 +27092,655 @@
         </is>
       </c>
     </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C453" t="n">
+        <v>743.5700000000001</v>
+      </c>
+      <c r="D453" t="n">
+        <v>-0.0033</v>
+      </c>
+      <c r="E453" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="F453" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K453" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>RVol: 0.86x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C454" t="n">
+        <v>228.52</v>
+      </c>
+      <c r="D454" t="n">
+        <v>0.0097</v>
+      </c>
+      <c r="E454" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="F454" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K454" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C455" t="n">
+        <v>341.27</v>
+      </c>
+      <c r="D455" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="E455" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="F455" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K455" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>RVol: 1.04x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C456" t="n">
+        <v>543.45</v>
+      </c>
+      <c r="D456" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="E456" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="F456" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K456" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C457" t="n">
+        <v>258.58</v>
+      </c>
+      <c r="D457" t="n">
+        <v>-0.0037</v>
+      </c>
+      <c r="E457" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="F457" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K457" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>RVol: 0.68x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C458" t="n">
+        <v>762.5</v>
+      </c>
+      <c r="D458" t="n">
+        <v>0.0263</v>
+      </c>
+      <c r="E458" t="n">
+        <v>36.43</v>
+      </c>
+      <c r="F458" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K458" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>RVol: 1.03x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C459" t="n">
+        <v>353.78</v>
+      </c>
+      <c r="D459" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="E459" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="F459" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K459" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C460" t="n">
+        <v>375.23</v>
+      </c>
+      <c r="D460" t="n">
+        <v>-0.0074</v>
+      </c>
+      <c r="E460" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="F460" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K460" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>RVol: 0.52x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>953.1900000000001</v>
+      </c>
+      <c r="D461" t="n">
+        <v>-0.0362</v>
+      </c>
+      <c r="E461" t="n">
+        <v>24.57</v>
+      </c>
+      <c r="F461" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K461" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>RVol: 1.13x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C462" t="n">
+        <v>380.71</v>
+      </c>
+      <c r="D462" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="E462" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="F462" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>RVol: 1.40x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C463" t="n">
+        <v>747.2</v>
+      </c>
+      <c r="D463" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="E463" t="n">
+        <v>55.07</v>
+      </c>
+      <c r="F463" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>RVol: 1.45x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-15
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M463"/>
+  <dimension ref="A1:M474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27741,6 +27741,655 @@
         </is>
       </c>
     </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C464" t="n">
+        <v>728.95</v>
+      </c>
+      <c r="D464" t="n">
+        <v>-0.0197</v>
+      </c>
+      <c r="E464" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="F464" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>RVol: 1.49x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C465" t="n">
+        <v>221.3</v>
+      </c>
+      <c r="D465" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="E465" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="F465" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C466" t="n">
+        <v>342.96</v>
+      </c>
+      <c r="D466" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E466" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="F466" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>RVol: 1.33x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C467" t="n">
+        <v>533.6900000000001</v>
+      </c>
+      <c r="D467" t="n">
+        <v>-0.018</v>
+      </c>
+      <c r="E467" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="F467" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>RVol: 0.96x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C468" t="n">
+        <v>254.08</v>
+      </c>
+      <c r="D468" t="n">
+        <v>-0.0174</v>
+      </c>
+      <c r="E468" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F468" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C469" t="n">
+        <v>737.54</v>
+      </c>
+      <c r="D469" t="n">
+        <v>-0.0327</v>
+      </c>
+      <c r="E469" t="n">
+        <v>27.21</v>
+      </c>
+      <c r="F469" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C470" t="n">
+        <v>347.64</v>
+      </c>
+      <c r="D470" t="n">
+        <v>-0.0174</v>
+      </c>
+      <c r="E470" t="n">
+        <v>13.06</v>
+      </c>
+      <c r="F470" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C471" t="n">
+        <v>367.16</v>
+      </c>
+      <c r="D471" t="n">
+        <v>-0.0215</v>
+      </c>
+      <c r="E471" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="F471" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C472" t="n">
+        <v>914.13</v>
+      </c>
+      <c r="D472" t="n">
+        <v>-0.04099999999999999</v>
+      </c>
+      <c r="E472" t="n">
+        <v>35.86</v>
+      </c>
+      <c r="F472" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>RVol: 1.02x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C473" t="n">
+        <v>364.1</v>
+      </c>
+      <c r="D473" t="n">
+        <v>-0.0436</v>
+      </c>
+      <c r="E473" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="F473" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C474" t="n">
+        <v>713.54</v>
+      </c>
+      <c r="D474" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="E474" t="n">
+        <v>40.18</v>
+      </c>
+      <c r="F474" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-16
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M474"/>
+  <dimension ref="A1:M485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28390,6 +28390,655 @@
         </is>
       </c>
     </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C475" t="n">
+        <v>728</v>
+      </c>
+      <c r="D475" t="n">
+        <v>-0.0013</v>
+      </c>
+      <c r="E475" t="n">
+        <v>14</v>
+      </c>
+      <c r="F475" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>RVol: 1.42x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C476" t="n">
+        <v>217.23</v>
+      </c>
+      <c r="D476" t="n">
+        <v>-0.0184</v>
+      </c>
+      <c r="E476" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="F476" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>RVol: 1.18x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C477" t="n">
+        <v>342</v>
+      </c>
+      <c r="D477" t="n">
+        <v>-0.0028</v>
+      </c>
+      <c r="E477" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F477" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>RVol: 1.04x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C478" t="n">
+        <v>539.4400000000001</v>
+      </c>
+      <c r="D478" t="n">
+        <v>0.0108</v>
+      </c>
+      <c r="E478" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="F478" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>RVol: 1.04x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C479" t="n">
+        <v>254.76</v>
+      </c>
+      <c r="D479" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="E479" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="F479" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C480" t="n">
+        <v>736.72</v>
+      </c>
+      <c r="D480" t="n">
+        <v>-0.0011</v>
+      </c>
+      <c r="E480" t="n">
+        <v>28.39</v>
+      </c>
+      <c r="F480" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C481" t="n">
+        <v>349.22</v>
+      </c>
+      <c r="D481" t="n">
+        <v>0.004500000000000001</v>
+      </c>
+      <c r="E481" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="F481" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C482" t="n">
+        <v>362.44</v>
+      </c>
+      <c r="D482" t="n">
+        <v>-0.0129</v>
+      </c>
+      <c r="E482" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="F482" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C483" t="n">
+        <v>931.24</v>
+      </c>
+      <c r="D483" t="n">
+        <v>0.0187</v>
+      </c>
+      <c r="E483" t="n">
+        <v>73.65000000000001</v>
+      </c>
+      <c r="F483" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>RVol: 1.45x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C484" t="n">
+        <v>356.45</v>
+      </c>
+      <c r="D484" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="E484" t="n">
+        <v>20.83</v>
+      </c>
+      <c r="F484" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>RVol: 1.35x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>690.8099999999999</v>
+      </c>
+      <c r="D485" t="n">
+        <v>-0.0319</v>
+      </c>
+      <c r="E485" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="F485" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>RVol: 1.20x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-17
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M485"/>
+  <dimension ref="A1:M496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29039,6 +29039,655 @@
         </is>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>709.8</v>
+      </c>
+      <c r="D486" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="E486" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="F486" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>RVol: 1.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>214.13</v>
+      </c>
+      <c r="D487" t="n">
+        <v>-0.0143</v>
+      </c>
+      <c r="E487" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="F487" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M487" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C488" t="n">
+        <v>343.46</v>
+      </c>
+      <c r="D488" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="E488" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="F488" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M488" t="inlineStr">
+        <is>
+          <t>RVol: 1.56x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C489" t="n">
+        <v>529.05</v>
+      </c>
+      <c r="D489" t="n">
+        <v>-0.0193</v>
+      </c>
+      <c r="E489" t="n">
+        <v>19.39</v>
+      </c>
+      <c r="F489" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M489" t="inlineStr">
+        <is>
+          <t>RVol: 1.03x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C490" t="n">
+        <v>250</v>
+      </c>
+      <c r="D490" t="n">
+        <v>-0.0187</v>
+      </c>
+      <c r="E490" t="n">
+        <v>6.94</v>
+      </c>
+      <c r="F490" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M490" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C491" t="n">
+        <v>709.3200000000001</v>
+      </c>
+      <c r="D491" t="n">
+        <v>-0.0372</v>
+      </c>
+      <c r="E491" t="n">
+        <v>35.78</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M491" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C492" t="n">
+        <v>340.59</v>
+      </c>
+      <c r="D492" t="n">
+        <v>-0.0247</v>
+      </c>
+      <c r="E492" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="F492" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M492" t="inlineStr">
+        <is>
+          <t>RVol: 1.08x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C493" t="n">
+        <v>354.72</v>
+      </c>
+      <c r="D493" t="n">
+        <v>-0.0213</v>
+      </c>
+      <c r="E493" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="F493" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M493" t="inlineStr">
+        <is>
+          <t>RVol: 1.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C494" t="n">
+        <v>878.84</v>
+      </c>
+      <c r="D494" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="E494" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="F494" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M494" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C495" t="n">
+        <v>332</v>
+      </c>
+      <c r="D495" t="n">
+        <v>-0.06860000000000001</v>
+      </c>
+      <c r="E495" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="F495" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M495" t="inlineStr">
+        <is>
+          <t>RVol: 0.86x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C496" t="n">
+        <v>639.01</v>
+      </c>
+      <c r="D496" t="n">
+        <v>-0.075</v>
+      </c>
+      <c r="E496" t="n">
+        <v>47.12</v>
+      </c>
+      <c r="F496" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M496" t="inlineStr">
+        <is>
+          <t>RVol: 1.24x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-20
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M496"/>
+  <dimension ref="A1:M507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29688,6 +29688,655 @@
         </is>
       </c>
     </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C497" t="n">
+        <v>718.36</v>
+      </c>
+      <c r="D497" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="E497" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="F497" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M497" t="inlineStr">
+        <is>
+          <t>RVol: 1.02x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C498" t="n">
+        <v>217.09</v>
+      </c>
+      <c r="D498" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="E498" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="F498" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M498" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C499" t="n">
+        <v>342.94</v>
+      </c>
+      <c r="D499" t="n">
+        <v>-0.0015</v>
+      </c>
+      <c r="E499" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="F499" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M499" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C500" t="n">
+        <v>533.52</v>
+      </c>
+      <c r="D500" t="n">
+        <v>0.008399999999999999</v>
+      </c>
+      <c r="E500" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M500" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C501" t="n">
+        <v>262.45</v>
+      </c>
+      <c r="D501" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="E501" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F501" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M501" t="inlineStr">
+        <is>
+          <t>RVol: 1.53x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C502" t="n">
+        <v>705.4400000000001</v>
+      </c>
+      <c r="D502" t="n">
+        <v>-0.005500000000000001</v>
+      </c>
+      <c r="E502" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="F502" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M502" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C503" t="n">
+        <v>344.18</v>
+      </c>
+      <c r="D503" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="E503" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M503" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C504" t="n">
+        <v>368.06</v>
+      </c>
+      <c r="D504" t="n">
+        <v>0.03759999999999999</v>
+      </c>
+      <c r="E504" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="F504" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr">
+        <is>
+          <t>RVol: 1.12x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C505" t="n">
+        <v>904.9</v>
+      </c>
+      <c r="D505" t="n">
+        <v>0.0297</v>
+      </c>
+      <c r="E505" t="n">
+        <v>26.24</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M505" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C506" t="n">
+        <v>352.21</v>
+      </c>
+      <c r="D506" t="n">
+        <v>0.0609</v>
+      </c>
+      <c r="E506" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M506" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C507" t="n">
+        <v>660.8099999999999</v>
+      </c>
+      <c r="D507" t="n">
+        <v>0.0341</v>
+      </c>
+      <c r="E507" t="n">
+        <v>21.19</v>
+      </c>
+      <c r="F507" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K507" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M507" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-21
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M507"/>
+  <dimension ref="A1:M518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30337,6 +30337,655 @@
         </is>
       </c>
     </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C508" t="n">
+        <v>717.63</v>
+      </c>
+      <c r="D508" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="E508" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="F508" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M508" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C509" t="n">
+        <v>216.47</v>
+      </c>
+      <c r="D509" t="n">
+        <v>-0.0029</v>
+      </c>
+      <c r="E509" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="F509" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M509" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C510" t="n">
+        <v>339.5</v>
+      </c>
+      <c r="D510" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="E510" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="F510" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M510" t="inlineStr">
+        <is>
+          <t>RVol: 0.96x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C511" t="n">
+        <v>531.87</v>
+      </c>
+      <c r="D511" t="n">
+        <v>-0.0031</v>
+      </c>
+      <c r="E511" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="F511" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M511" t="inlineStr">
+        <is>
+          <t>RVol: 0.66x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C512" t="n">
+        <v>262.63</v>
+      </c>
+      <c r="D512" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="E512" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="F512" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M512" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C513" t="n">
+        <v>694.25</v>
+      </c>
+      <c r="D513" t="n">
+        <v>-0.0159</v>
+      </c>
+      <c r="E513" t="n">
+        <v>15.46</v>
+      </c>
+      <c r="F513" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K513" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M513" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C514" t="n">
+        <v>340.28</v>
+      </c>
+      <c r="D514" t="n">
+        <v>-0.0113</v>
+      </c>
+      <c r="E514" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="F514" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M514" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C515" t="n">
+        <v>373.71</v>
+      </c>
+      <c r="D515" t="n">
+        <v>0.0154</v>
+      </c>
+      <c r="E515" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="F515" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K515" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C516" t="n">
+        <v>896.0700000000001</v>
+      </c>
+      <c r="D516" t="n">
+        <v>-0.0098</v>
+      </c>
+      <c r="E516" t="n">
+        <v>37.37</v>
+      </c>
+      <c r="F516" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M516" t="inlineStr">
+        <is>
+          <t>RVol: 0.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C517" t="n">
+        <v>364.32</v>
+      </c>
+      <c r="D517" t="n">
+        <v>0.0344</v>
+      </c>
+      <c r="E517" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F517" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K517" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M517" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C518" t="n">
+        <v>675.13</v>
+      </c>
+      <c r="D518" t="n">
+        <v>0.0217</v>
+      </c>
+      <c r="E518" t="n">
+        <v>38.28</v>
+      </c>
+      <c r="F518" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M518" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-22
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M518"/>
+  <dimension ref="A1:M529"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30986,6 +30986,655 @@
         </is>
       </c>
     </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>725.2</v>
+      </c>
+      <c r="D519" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="E519" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F519" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M519" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C520" t="n">
+        <v>221.97</v>
+      </c>
+      <c r="D520" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="E520" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="F520" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M520" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C521" t="n">
+        <v>343.99</v>
+      </c>
+      <c r="D521" t="n">
+        <v>0.0132</v>
+      </c>
+      <c r="E521" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="F521" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K521" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M521" t="inlineStr">
+        <is>
+          <t>RVol: 0.96x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C522" t="n">
+        <v>532.95</v>
+      </c>
+      <c r="D522" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="E522" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="F522" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M522" t="inlineStr">
+        <is>
+          <t>RVol: 0.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C523" t="n">
+        <v>262.37</v>
+      </c>
+      <c r="D523" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="E523" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="F523" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K523" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M523" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C524" t="n">
+        <v>697.52</v>
+      </c>
+      <c r="D524" t="n">
+        <v>0.004699999999999999</v>
+      </c>
+      <c r="E524" t="n">
+        <v>23.54</v>
+      </c>
+      <c r="F524" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K524" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L524" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M524" t="inlineStr">
+        <is>
+          <t>RVol: 1.25x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C525" t="n">
+        <v>334.76</v>
+      </c>
+      <c r="D525" t="n">
+        <v>-0.0162</v>
+      </c>
+      <c r="E525" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="F525" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K525" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L525" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M525" t="inlineStr">
+        <is>
+          <t>RVol: 1.18x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C526" t="n">
+        <v>386.47</v>
+      </c>
+      <c r="D526" t="n">
+        <v>0.0341</v>
+      </c>
+      <c r="E526" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="F526" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K526" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L526" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M526" t="inlineStr">
+        <is>
+          <t>RVol: 1.26x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C527" t="n">
+        <v>913.67</v>
+      </c>
+      <c r="D527" t="n">
+        <v>0.0196</v>
+      </c>
+      <c r="E527" t="n">
+        <v>39</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K527" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L527" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M527" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C528" t="n">
+        <v>378.51</v>
+      </c>
+      <c r="D528" t="n">
+        <v>0.0389</v>
+      </c>
+      <c r="E528" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="F528" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M528" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C529" t="n">
+        <v>696.89</v>
+      </c>
+      <c r="D529" t="n">
+        <v>0.0322</v>
+      </c>
+      <c r="E529" t="n">
+        <v>32.91</v>
+      </c>
+      <c r="F529" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K529" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L529" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M529" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-23
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M529"/>
+  <dimension ref="A1:M540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31635,6 +31635,655 @@
         </is>
       </c>
     </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C530" t="n">
+        <v>704.47</v>
+      </c>
+      <c r="D530" t="n">
+        <v>-0.0286</v>
+      </c>
+      <c r="E530" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="F530" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K530" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L530" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M530" t="inlineStr">
+        <is>
+          <t>RVol: 1.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C531" t="n">
+        <v>212.21</v>
+      </c>
+      <c r="D531" t="n">
+        <v>-0.044</v>
+      </c>
+      <c r="E531" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="F531" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K531" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M531" t="inlineStr">
+        <is>
+          <t>RVol: 1.20x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C532" t="n">
+        <v>348.22</v>
+      </c>
+      <c r="D532" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="E532" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="F532" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K532" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M532" t="inlineStr">
+        <is>
+          <t>RVol: 1.18x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C533" t="n">
+        <v>521.08</v>
+      </c>
+      <c r="D533" t="n">
+        <v>-0.0223</v>
+      </c>
+      <c r="E533" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="F533" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K533" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L533" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M533" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C534" t="n">
+        <v>250.38</v>
+      </c>
+      <c r="D534" t="n">
+        <v>-0.0457</v>
+      </c>
+      <c r="E534" t="n">
+        <v>10.41</v>
+      </c>
+      <c r="F534" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K534" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L534" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M534" t="inlineStr">
+        <is>
+          <t>RVol: 1.36x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C535" t="n">
+        <v>648.85</v>
+      </c>
+      <c r="D535" t="n">
+        <v>-0.0698</v>
+      </c>
+      <c r="E535" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="F535" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K535" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M535" t="inlineStr">
+        <is>
+          <t>RVol: 2.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C536" t="n">
+        <v>324.22</v>
+      </c>
+      <c r="D536" t="n">
+        <v>-0.0315</v>
+      </c>
+      <c r="E536" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="F536" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K536" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L536" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M536" t="inlineStr">
+        <is>
+          <t>RVol: 1.15x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C537" t="n">
+        <v>374.58</v>
+      </c>
+      <c r="D537" t="n">
+        <v>-0.0308</v>
+      </c>
+      <c r="E537" t="n">
+        <v>15.15</v>
+      </c>
+      <c r="F537" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K537" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L537" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M537" t="inlineStr">
+        <is>
+          <t>RVol: 1.44x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C538" t="n">
+        <v>856.49</v>
+      </c>
+      <c r="D538" t="n">
+        <v>-0.0626</v>
+      </c>
+      <c r="E538" t="n">
+        <v>59.05</v>
+      </c>
+      <c r="F538" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K538" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L538" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M538" t="inlineStr">
+        <is>
+          <t>RVol: 1.17x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C539" t="n">
+        <v>354.19</v>
+      </c>
+      <c r="D539" t="n">
+        <v>-0.0643</v>
+      </c>
+      <c r="E539" t="n">
+        <v>19.11</v>
+      </c>
+      <c r="F539" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M539" t="inlineStr">
+        <is>
+          <t>RVol: 1.26x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C540" t="n">
+        <v>642.14</v>
+      </c>
+      <c r="D540" t="n">
+        <v>-0.0786</v>
+      </c>
+      <c r="E540" t="n">
+        <v>43.77</v>
+      </c>
+      <c r="F540" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M540" t="inlineStr">
+        <is>
+          <t>RVol: 1.15x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-24
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M540"/>
+  <dimension ref="A1:M551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32284,6 +32284,655 @@
         </is>
       </c>
     </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C541" t="n">
+        <v>704.4</v>
+      </c>
+      <c r="D541" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="E541" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="F541" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K541" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L541" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M541" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C542" t="n">
+        <v>210.96</v>
+      </c>
+      <c r="D542" t="n">
+        <v>-0.0059</v>
+      </c>
+      <c r="E542" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F542" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K542" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M542" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C543" t="n">
+        <v>347.72</v>
+      </c>
+      <c r="D543" t="n">
+        <v>-0.0014</v>
+      </c>
+      <c r="E543" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="F543" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K543" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M543" t="inlineStr">
+        <is>
+          <t>RVol: 1.04x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C544" t="n">
+        <v>524.51</v>
+      </c>
+      <c r="D544" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="E544" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F544" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K544" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M544" t="inlineStr">
+        <is>
+          <t>RVol: 0.62x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C545" t="n">
+        <v>248</v>
+      </c>
+      <c r="D545" t="n">
+        <v>-0.0095</v>
+      </c>
+      <c r="E545" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F545" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K545" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M545" t="inlineStr">
+        <is>
+          <t>RVol: 0.70x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C546" t="n">
+        <v>642.62</v>
+      </c>
+      <c r="D546" t="n">
+        <v>-0.009599999999999999</v>
+      </c>
+      <c r="E546" t="n">
+        <v>14.77</v>
+      </c>
+      <c r="F546" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L546" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M546" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C547" t="n">
+        <v>320.21</v>
+      </c>
+      <c r="D547" t="n">
+        <v>-0.0124</v>
+      </c>
+      <c r="E547" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="F547" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M547" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C548" t="n">
+        <v>372.22</v>
+      </c>
+      <c r="D548" t="n">
+        <v>-0.0063</v>
+      </c>
+      <c r="E548" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="F548" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L548" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M548" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C549" t="n">
+        <v>877.55</v>
+      </c>
+      <c r="D549" t="n">
+        <v>0.0246</v>
+      </c>
+      <c r="E549" t="n">
+        <v>33.55</v>
+      </c>
+      <c r="F549" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M549" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C550" t="n">
+        <v>343.67</v>
+      </c>
+      <c r="D550" t="n">
+        <v>-0.0297</v>
+      </c>
+      <c r="E550" t="n">
+        <v>21.11</v>
+      </c>
+      <c r="F550" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M550" t="inlineStr">
+        <is>
+          <t>RVol: 1.46x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C551" t="n">
+        <v>630.49</v>
+      </c>
+      <c r="D551" t="n">
+        <v>-0.0181</v>
+      </c>
+      <c r="E551" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="F551" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L551" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M551" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-27
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M551"/>
+  <dimension ref="A1:M562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32933,6 +32933,655 @@
         </is>
       </c>
     </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C552" t="n">
+        <v>712.2</v>
+      </c>
+      <c r="D552" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="E552" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F552" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M552" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C553" t="n">
+        <v>216</v>
+      </c>
+      <c r="D553" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="E553" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="F553" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K553" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M553" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C554" t="n">
+        <v>343.91</v>
+      </c>
+      <c r="D554" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="E554" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="F554" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K554" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M554" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C555" t="n">
+        <v>532.6</v>
+      </c>
+      <c r="D555" t="n">
+        <v>0.0154</v>
+      </c>
+      <c r="E555" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="F555" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K555" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M555" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C556" t="n">
+        <v>249.09</v>
+      </c>
+      <c r="D556" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="E556" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F556" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M556" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C557" t="n">
+        <v>630.5599999999999</v>
+      </c>
+      <c r="D557" t="n">
+        <v>-0.0188</v>
+      </c>
+      <c r="E557" t="n">
+        <v>19.89</v>
+      </c>
+      <c r="F557" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K557" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L557" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M557" t="inlineStr">
+        <is>
+          <t>RVol: 1.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C558" t="n">
+        <v>316.8</v>
+      </c>
+      <c r="D558" t="n">
+        <v>-0.0106</v>
+      </c>
+      <c r="E558" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="F558" t="n">
+        <v>1</v>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M558" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C559" t="n">
+        <v>391.62</v>
+      </c>
+      <c r="D559" t="n">
+        <v>0.0521</v>
+      </c>
+      <c r="E559" t="n">
+        <v>13.54</v>
+      </c>
+      <c r="F559" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M559" t="inlineStr">
+        <is>
+          <t>RVol: 1.45x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C560" t="n">
+        <v>903.7</v>
+      </c>
+      <c r="D560" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="E560" t="n">
+        <v>32.98</v>
+      </c>
+      <c r="F560" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M560" t="inlineStr">
+        <is>
+          <t>RVol: 0.84x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C561" t="n">
+        <v>356.13</v>
+      </c>
+      <c r="D561" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="E561" t="n">
+        <v>23.83</v>
+      </c>
+      <c r="F561" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M561" t="inlineStr">
+        <is>
+          <t>RVol: 0.98x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C562" t="n">
+        <v>644.21</v>
+      </c>
+      <c r="D562" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="E562" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="F562" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M562" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-28
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M562"/>
+  <dimension ref="A1:M573"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33582,6 +33582,655 @@
         </is>
       </c>
     </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C563" t="n">
+        <v>721.25</v>
+      </c>
+      <c r="D563" t="n">
+        <v>0.0127</v>
+      </c>
+      <c r="E563" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="F563" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M563" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C564" t="n">
+        <v>217.94</v>
+      </c>
+      <c r="D564" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="E564" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="F564" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M564" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C565" t="n">
+        <v>347.1</v>
+      </c>
+      <c r="D565" t="n">
+        <v>0.009300000000000001</v>
+      </c>
+      <c r="E565" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="F565" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K565" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M565" t="inlineStr">
+        <is>
+          <t>RVol: 0.98x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C566" t="n">
+        <v>531.33</v>
+      </c>
+      <c r="D566" t="n">
+        <v>-0.0024</v>
+      </c>
+      <c r="E566" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="F566" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M566" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C567" t="n">
+        <v>253.1</v>
+      </c>
+      <c r="D567" t="n">
+        <v>0.0161</v>
+      </c>
+      <c r="E567" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="F567" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M567" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C568" t="n">
+        <v>620.1900000000001</v>
+      </c>
+      <c r="D568" t="n">
+        <v>-0.0164</v>
+      </c>
+      <c r="E568" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="F568" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M568" t="inlineStr">
+        <is>
+          <t>RVol: 2.60x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C569" t="n">
+        <v>320.58</v>
+      </c>
+      <c r="D569" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="E569" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="F569" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M569" t="inlineStr">
+        <is>
+          <t>RVol: 1.19x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C570" t="n">
+        <v>407.46</v>
+      </c>
+      <c r="D570" t="n">
+        <v>0.0404</v>
+      </c>
+      <c r="E570" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F570" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M570" t="inlineStr">
+        <is>
+          <t>RVol: 1.21x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C571" t="n">
+        <v>928.76</v>
+      </c>
+      <c r="D571" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="E571" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="F571" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K571" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L571" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M571" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C572" t="n">
+        <v>380.88</v>
+      </c>
+      <c r="D572" t="n">
+        <v>0.06950000000000001</v>
+      </c>
+      <c r="E572" t="n">
+        <v>29.84</v>
+      </c>
+      <c r="F572" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M572" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C573" t="n">
+        <v>667.85</v>
+      </c>
+      <c r="D573" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="E573" t="n">
+        <v>39.11</v>
+      </c>
+      <c r="F573" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K573" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L573" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M573" t="inlineStr">
+        <is>
+          <t>RVol: 1.57x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-29
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M573"/>
+  <dimension ref="A1:M584"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34231,6 +34231,655 @@
         </is>
       </c>
     </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C574" t="n">
+        <v>725.61</v>
+      </c>
+      <c r="D574" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="E574" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="F574" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L574" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M574" t="inlineStr">
+        <is>
+          <t>RVol: 0.84x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C575" t="n">
+        <v>215.38</v>
+      </c>
+      <c r="D575" t="n">
+        <v>-0.0117</v>
+      </c>
+      <c r="E575" t="n">
+        <v>5.52</v>
+      </c>
+      <c r="F575" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K575" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L575" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M575" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C576" t="n">
+        <v>343.83</v>
+      </c>
+      <c r="D576" t="n">
+        <v>-0.009399999999999999</v>
+      </c>
+      <c r="E576" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="F576" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K576" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L576" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M576" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C577" t="n">
+        <v>531.01</v>
+      </c>
+      <c r="D577" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="E577" t="n">
+        <v>8.869999999999999</v>
+      </c>
+      <c r="F577" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K577" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L577" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M577" t="inlineStr">
+        <is>
+          <t>RVol: 1.42x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C578" t="n">
+        <v>254.6</v>
+      </c>
+      <c r="D578" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="E578" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="F578" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K578" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L578" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M578" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C579" t="n">
+        <v>612.49</v>
+      </c>
+      <c r="D579" t="n">
+        <v>-0.0124</v>
+      </c>
+      <c r="E579" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="F579" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K579" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L579" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M579" t="inlineStr">
+        <is>
+          <t>RVol: 1.69x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C580" t="n">
+        <v>324.89</v>
+      </c>
+      <c r="D580" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="E580" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F580" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K580" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L580" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M580" t="inlineStr">
+        <is>
+          <t>RVol: 2.05x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C581" t="n">
+        <v>404.22</v>
+      </c>
+      <c r="D581" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="E581" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="F581" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K581" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L581" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M581" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C582" t="n">
+        <v>983.23</v>
+      </c>
+      <c r="D582" t="n">
+        <v>0.05860000000000001</v>
+      </c>
+      <c r="E582" t="n">
+        <v>30.66</v>
+      </c>
+      <c r="F582" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K582" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L582" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M582" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C583" t="n">
+        <v>396.42</v>
+      </c>
+      <c r="D583" t="n">
+        <v>0.0408</v>
+      </c>
+      <c r="E583" t="n">
+        <v>22.44</v>
+      </c>
+      <c r="F583" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K583" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L583" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M583" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C584" t="n">
+        <v>697.97</v>
+      </c>
+      <c r="D584" t="n">
+        <v>0.0451</v>
+      </c>
+      <c r="E584" t="n">
+        <v>77.44</v>
+      </c>
+      <c r="F584" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K584" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L584" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M584" t="inlineStr">
+        <is>
+          <t>RVol: 1.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-30
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M584"/>
+  <dimension ref="A1:M595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34880,6 +34880,655 @@
         </is>
       </c>
     </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C585" t="n">
+        <v>715.34</v>
+      </c>
+      <c r="D585" t="n">
+        <v>-0.0142</v>
+      </c>
+      <c r="E585" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="F585" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K585" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L585" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M585" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C586" t="n">
+        <v>213.66</v>
+      </c>
+      <c r="D586" t="n">
+        <v>-0.008</v>
+      </c>
+      <c r="E586" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F586" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K586" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L586" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M586" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C587" t="n">
+        <v>348.91</v>
+      </c>
+      <c r="D587" t="n">
+        <v>0.0148</v>
+      </c>
+      <c r="E587" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="F587" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K587" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L587" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M587" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C588" t="n">
+        <v>530.14</v>
+      </c>
+      <c r="D588" t="n">
+        <v>-0.0016</v>
+      </c>
+      <c r="E588" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="F588" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K588" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L588" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M588" t="inlineStr">
+        <is>
+          <t>RVol: 1.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C589" t="n">
+        <v>243.79</v>
+      </c>
+      <c r="D589" t="n">
+        <v>-0.0425</v>
+      </c>
+      <c r="E589" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="F589" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K589" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L589" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M589" t="inlineStr">
+        <is>
+          <t>RVol: 2.40x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C590" t="n">
+        <v>624.52</v>
+      </c>
+      <c r="D590" t="n">
+        <v>0.0196</v>
+      </c>
+      <c r="E590" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="F590" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L590" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M590" t="inlineStr">
+        <is>
+          <t>RVol: 1.45x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C591" t="n">
+        <v>283.82</v>
+      </c>
+      <c r="D591" t="n">
+        <v>-0.1264</v>
+      </c>
+      <c r="E591" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="F591" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K591" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L591" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M591" t="inlineStr">
+        <is>
+          <t>RVol: 5.35x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C592" t="n">
+        <v>403.3</v>
+      </c>
+      <c r="D592" t="n">
+        <v>-0.0023</v>
+      </c>
+      <c r="E592" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L592" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M592" t="inlineStr">
+        <is>
+          <t>RVol: 0.61x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C593" t="n">
+        <v>934.27</v>
+      </c>
+      <c r="D593" t="n">
+        <v>-0.0498</v>
+      </c>
+      <c r="E593" t="n">
+        <v>43.77</v>
+      </c>
+      <c r="F593" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K593" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L593" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M593" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C594" t="n">
+        <v>395.41</v>
+      </c>
+      <c r="D594" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="E594" t="n">
+        <v>13.87</v>
+      </c>
+      <c r="F594" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K594" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L594" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M594" t="inlineStr">
+        <is>
+          <t>RVol: 0.56x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C595" t="n">
+        <v>700.47</v>
+      </c>
+      <c r="D595" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="E595" t="n">
+        <v>43.24</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L595" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M595" t="inlineStr">
+        <is>
+          <t>RVol: 0.91x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-10-31
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M595"/>
+  <dimension ref="A1:M606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35529,6 +35529,655 @@
         </is>
       </c>
     </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C596" t="n">
+        <v>690.49</v>
+      </c>
+      <c r="D596" t="n">
+        <v>-0.0347</v>
+      </c>
+      <c r="E596" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="F596" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L596" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M596" t="inlineStr">
+        <is>
+          <t>RVol: 2.32x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C597" t="n">
+        <v>204.64</v>
+      </c>
+      <c r="D597" t="n">
+        <v>-0.04219999999999999</v>
+      </c>
+      <c r="E597" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="F597" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K597" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L597" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M597" t="inlineStr">
+        <is>
+          <t>RVol: 1.67x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C598" t="n">
+        <v>344.63</v>
+      </c>
+      <c r="D598" t="n">
+        <v>-0.0123</v>
+      </c>
+      <c r="E598" t="n">
+        <v>14.84</v>
+      </c>
+      <c r="F598" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L598" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M598" t="inlineStr">
+        <is>
+          <t>RVol: 1.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C599" t="n">
+        <v>521.91</v>
+      </c>
+      <c r="D599" t="n">
+        <v>-0.0155</v>
+      </c>
+      <c r="E599" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="F599" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K599" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L599" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M599" t="inlineStr">
+        <is>
+          <t>RVol: 1.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C600" t="n">
+        <v>240.35</v>
+      </c>
+      <c r="D600" t="n">
+        <v>-0.0141</v>
+      </c>
+      <c r="E600" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="F600" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K600" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L600" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M600" t="inlineStr">
+        <is>
+          <t>RVol: 2.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C601" t="n">
+        <v>614.99</v>
+      </c>
+      <c r="D601" t="n">
+        <v>-0.0153</v>
+      </c>
+      <c r="E601" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="F601" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K601" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L601" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M601" t="inlineStr">
+        <is>
+          <t>RVol: 1.13x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C602" t="n">
+        <v>279.84</v>
+      </c>
+      <c r="D602" t="n">
+        <v>-0.014</v>
+      </c>
+      <c r="E602" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="F602" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K602" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L602" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M602" t="inlineStr">
+        <is>
+          <t>RVol: 2.08x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C603" t="n">
+        <v>399.81</v>
+      </c>
+      <c r="D603" t="n">
+        <v>-0.008699999999999999</v>
+      </c>
+      <c r="E603" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="F603" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K603" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L603" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M603" t="inlineStr">
+        <is>
+          <t>RVol: 1.13x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C604" t="n">
+        <v>884.74</v>
+      </c>
+      <c r="D604" t="n">
+        <v>-0.053</v>
+      </c>
+      <c r="E604" t="n">
+        <v>44.95</v>
+      </c>
+      <c r="F604" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K604" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L604" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M604" t="inlineStr">
+        <is>
+          <t>RVol: 1.19x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C605" t="n">
+        <v>366.11</v>
+      </c>
+      <c r="D605" t="n">
+        <v>-0.0741</v>
+      </c>
+      <c r="E605" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="F605" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K605" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L605" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M605" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C606" t="n">
+        <v>644.58</v>
+      </c>
+      <c r="D606" t="n">
+        <v>-0.07980000000000001</v>
+      </c>
+      <c r="E606" t="n">
+        <v>53.19</v>
+      </c>
+      <c r="F606" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K606" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L606" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M606" t="inlineStr">
+        <is>
+          <t>RVol: 0.96x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>